<commit_message>
Update core portal logic, templates, and analytics dashboard
</commit_message>
<xml_diff>
--- a/Comparision Format Sheet.xlsx
+++ b/Comparision Format Sheet.xlsx
@@ -143,7 +143,7 @@
     <numFmt numFmtId="180" formatCode="[$-1010407]dddd\,\ dd\.\ mmmm\ yyyy;@"/>
     <numFmt numFmtId="181" formatCode="&quot;₹&quot;#,##0"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="25">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -185,13 +185,6 @@
       <color rgb="FF000000"/>
       <name val="Microsoft YaHei"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -586,7 +579,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="70">
+  <borders count="66">
     <border>
       <left/>
       <right/>
@@ -788,9 +781,141 @@
         <color auto="1"/>
       </left>
       <right/>
-      <top/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
       <bottom style="thin">
         <color rgb="FFD9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
       </bottom>
       <diagonal/>
     </border>
@@ -815,115 +940,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top style="medium">
@@ -934,17 +950,6 @@
     </border>
     <border>
       <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="medium">
         <color auto="1"/>
       </right>
@@ -985,7 +990,52 @@
       <right style="thin">
         <color auto="1"/>
       </right>
-      <top style="medium">
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
         <color auto="1"/>
       </top>
       <bottom/>
@@ -998,7 +1048,7 @@
       <right style="thin">
         <color auto="1"/>
       </right>
-      <top style="medium">
+      <top style="thin">
         <color auto="1"/>
       </top>
       <bottom/>
@@ -1011,7 +1061,60 @@
       <right style="medium">
         <color auto="1"/>
       </right>
-      <top style="medium">
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
         <color auto="1"/>
       </top>
       <bottom/>
@@ -1022,22 +1125,53 @@
       <right style="thin">
         <color auto="1"/>
       </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
       <top style="medium">
         <color auto="1"/>
       </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="medium">
+      <left/>
+      <right/>
+      <top style="thin">
         <color auto="1"/>
       </top>
       <bottom style="thin">
@@ -1046,40 +1180,8 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
+      <left/>
       <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
         <color auto="1"/>
       </right>
       <top style="thin">
@@ -1104,52 +1206,26 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="medium">
         <color auto="1"/>
       </right>
       <top style="thin">
         <color auto="1"/>
       </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
       <bottom style="medium">
         <color auto="1"/>
       </bottom>
@@ -1165,10 +1241,8 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
+      <left/>
+      <right style="medium">
         <color auto="1"/>
       </right>
       <top/>
@@ -1179,7 +1253,7 @@
     </border>
     <border>
       <left/>
-      <right style="medium">
+      <right style="thin">
         <color auto="1"/>
       </right>
       <top/>
@@ -1189,151 +1263,26 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
       <right style="medium">
         <color auto="1"/>
       </right>
       <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
       <bottom style="medium">
         <color auto="1"/>
       </bottom>
@@ -1440,152 +1389,152 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="58" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="62" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="63" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="63" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="64" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="12" borderId="65" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="13" borderId="66" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="65" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="14" borderId="67" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="68" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="69" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="59" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="59" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="60" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="61" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="62" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="61" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="14" borderId="63" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="64" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="65" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="99">
+  <cellXfs count="101">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1675,18 +1624,24 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1699,13 +1654,13 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1714,7 +1669,28 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="181" fontId="4" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="4" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="4" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="181" fontId="4" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1723,160 +1699,139 @@
     <xf numFmtId="181" fontId="4" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="4" fillId="9" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="4" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="4" fillId="9" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="181" fontId="4" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="181" fontId="4" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="181" fontId="4" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="181" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="181" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="181" fontId="4" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="181" fontId="4" fillId="9" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="181" fontId="4" fillId="0" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="4" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="181" fontId="4" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="181" fontId="4" fillId="9" borderId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="181" fontId="4" fillId="0" borderId="48" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="4" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="3" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="3" fillId="9" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="3" fillId="9" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="3" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="181" fontId="4" fillId="0" borderId="52" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="181" fontId="4" fillId="0" borderId="54" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="181" fontId="4" fillId="0" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="181" fontId="4" fillId="0" borderId="53" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="181" fontId="3" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="181" fontId="3" fillId="9" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="181" fontId="3" fillId="9" borderId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="181" fontId="3" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2225,11 +2180,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:S25"/>
+  <dimension ref="A1:S27"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.2" style="1" customWidth="1"/>
-    <col min="2" max="2" width="25.4285714285714" style="1" customWidth="1"/>
+    <col min="2" max="2" width="32.7142857142857" style="1" customWidth="1"/>
     <col min="3" max="3" width="10.1428571428571" style="1" customWidth="1"/>
     <col min="4" max="4" width="12.2857142857143" style="1" customWidth="1"/>
     <col min="5" max="11" width="15.5809523809524" style="1" customWidth="1"/>
@@ -2352,132 +2307,132 @@
     </row>
     <row r="5" s="1" customFormat="1" ht="31.25" customHeight="1" spans="1:19">
       <c r="A5" s="31"/>
-      <c r="B5" s="21"/>
-      <c r="C5" s="21"/>
-      <c r="D5" s="22"/>
-      <c r="E5" s="32" t="s">
+      <c r="B5" s="32"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="33"/>
+      <c r="E5" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="33"/>
-      <c r="G5" s="34"/>
-      <c r="H5" s="33" t="s">
+      <c r="F5" s="35"/>
+      <c r="G5" s="36"/>
+      <c r="H5" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I5" s="33"/>
-      <c r="J5" s="34"/>
-      <c r="K5" s="33" t="s">
+      <c r="I5" s="35"/>
+      <c r="J5" s="36"/>
+      <c r="K5" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="L5" s="33"/>
-      <c r="M5" s="35"/>
-      <c r="N5" s="33" t="s">
+      <c r="L5" s="35"/>
+      <c r="M5" s="37"/>
+      <c r="N5" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="O5" s="33"/>
-      <c r="P5" s="35"/>
-      <c r="Q5" s="33" t="s">
+      <c r="O5" s="35"/>
+      <c r="P5" s="37"/>
+      <c r="Q5" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="R5" s="33"/>
-      <c r="S5" s="35"/>
+      <c r="R5" s="35"/>
+      <c r="S5" s="37"/>
     </row>
     <row r="6" s="1" customFormat="1" ht="37" customHeight="1" spans="1:19">
-      <c r="A6" s="36"/>
-      <c r="B6" s="37"/>
-      <c r="C6" s="37"/>
-      <c r="D6" s="38"/>
-      <c r="E6" s="39" t="s">
+      <c r="A6" s="38"/>
+      <c r="B6" s="39"/>
+      <c r="C6" s="39"/>
+      <c r="D6" s="40"/>
+      <c r="E6" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="F6" s="40" t="s">
+      <c r="F6" s="42" t="s">
         <v>17</v>
       </c>
-      <c r="G6" s="40" t="s">
+      <c r="G6" s="42" t="s">
         <v>18</v>
       </c>
-      <c r="H6" s="40" t="s">
+      <c r="H6" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="I6" s="40" t="s">
+      <c r="I6" s="42" t="s">
         <v>17</v>
       </c>
-      <c r="J6" s="40" t="s">
+      <c r="J6" s="42" t="s">
         <v>18</v>
       </c>
-      <c r="K6" s="40" t="s">
+      <c r="K6" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="L6" s="40" t="s">
+      <c r="L6" s="42" t="s">
         <v>17</v>
       </c>
-      <c r="M6" s="41" t="s">
+      <c r="M6" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="N6" s="40" t="s">
+      <c r="N6" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="O6" s="40" t="s">
+      <c r="O6" s="42" t="s">
         <v>17</v>
       </c>
-      <c r="P6" s="41" t="s">
+      <c r="P6" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="Q6" s="40" t="s">
+      <c r="Q6" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="R6" s="40" t="s">
+      <c r="R6" s="42" t="s">
         <v>17</v>
       </c>
-      <c r="S6" s="41" t="s">
+      <c r="S6" s="43" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="7" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A7" s="42">
+      <c r="A7" s="44">
         <v>1</v>
       </c>
-      <c r="B7" s="43"/>
-      <c r="C7" s="43"/>
-      <c r="D7" s="43"/>
-      <c r="E7" s="44"/>
-      <c r="F7" s="45"/>
-      <c r="G7" s="45">
+      <c r="B7" s="45"/>
+      <c r="C7" s="45"/>
+      <c r="D7" s="45"/>
+      <c r="E7" s="46"/>
+      <c r="F7" s="46"/>
+      <c r="G7" s="46">
         <f t="shared" ref="G7:G9" si="0">IF(F7&gt;0,C7*F7,IF(E7&gt;0,C7*E7,0))</f>
         <v>0</v>
       </c>
-      <c r="H7" s="45"/>
-      <c r="I7" s="45"/>
-      <c r="J7" s="45">
+      <c r="H7" s="46"/>
+      <c r="I7" s="46"/>
+      <c r="J7" s="46">
         <f t="shared" ref="J7:J9" si="1">IF(I7&gt;0,C7*I7,IF(H7&gt;0,C7*H7,0))</f>
         <v>0</v>
       </c>
-      <c r="K7" s="45"/>
-      <c r="L7" s="45"/>
+      <c r="K7" s="46"/>
+      <c r="L7" s="46"/>
       <c r="M7" s="46">
-        <f t="shared" ref="M7:M9" si="2">IF(L7&gt;0,C7*L7,IF(K7&gt;0,C7*K7,0))</f>
-        <v>0</v>
-      </c>
-      <c r="N7" s="45"/>
-      <c r="O7" s="45"/>
+        <f t="shared" ref="M7:M10" si="2">IF(L7&gt;0,C7*L7,IF(K7&gt;0,C7*K7,0))</f>
+        <v>0</v>
+      </c>
+      <c r="N7" s="46"/>
+      <c r="O7" s="46"/>
       <c r="P7" s="46">
         <f t="shared" ref="P7:P9" si="3">IF(O7&gt;0,C7*O7,IF(N7&gt;0,C7*N7,0))</f>
         <v>0</v>
       </c>
-      <c r="Q7" s="45"/>
-      <c r="R7" s="45"/>
-      <c r="S7" s="46">
+      <c r="Q7" s="46"/>
+      <c r="R7" s="46"/>
+      <c r="S7" s="47">
         <f t="shared" ref="S7:S9" si="4">IF(R7&gt;0,C7*R7,IF(Q7&gt;0,C7*Q7,0))</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A8" s="47">
+      <c r="A8" s="48">
         <v>2</v>
       </c>
-      <c r="B8" s="48"/>
-      <c r="C8" s="48"/>
-      <c r="D8" s="48"/>
-      <c r="E8" s="49"/>
+      <c r="B8" s="49"/>
+      <c r="C8" s="49"/>
+      <c r="D8" s="49"/>
+      <c r="E8" s="50"/>
       <c r="F8" s="50"/>
       <c r="G8" s="50">
         <f t="shared" si="0"/>
@@ -2491,19 +2446,19 @@
       </c>
       <c r="K8" s="50"/>
       <c r="L8" s="50"/>
-      <c r="M8" s="51">
+      <c r="M8" s="50">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="N8" s="50"/>
       <c r="O8" s="50"/>
-      <c r="P8" s="51">
+      <c r="P8" s="50">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="Q8" s="50"/>
       <c r="R8" s="50"/>
-      <c r="S8" s="46">
+      <c r="S8" s="51">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
@@ -2515,434 +2470,510 @@
       <c r="B9" s="53"/>
       <c r="C9" s="53"/>
       <c r="D9" s="53"/>
-      <c r="E9" s="54"/>
-      <c r="F9" s="55"/>
-      <c r="G9" s="55">
+      <c r="E9" s="50"/>
+      <c r="F9" s="50"/>
+      <c r="G9" s="50">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H9" s="55"/>
-      <c r="I9" s="55"/>
-      <c r="J9" s="55">
+      <c r="H9" s="50"/>
+      <c r="I9" s="50"/>
+      <c r="J9" s="50">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="K9" s="55"/>
-      <c r="L9" s="55"/>
-      <c r="M9" s="56">
+      <c r="K9" s="50"/>
+      <c r="L9" s="50"/>
+      <c r="M9" s="50">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="N9" s="55"/>
-      <c r="O9" s="55"/>
-      <c r="P9" s="56">
+      <c r="N9" s="50"/>
+      <c r="O9" s="50"/>
+      <c r="P9" s="50">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="Q9" s="55"/>
-      <c r="R9" s="55"/>
-      <c r="S9" s="56">
+      <c r="Q9" s="50"/>
+      <c r="R9" s="50"/>
+      <c r="S9" s="51">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
     <row r="10" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A10" s="57" t="s">
-        <v>19</v>
-      </c>
-      <c r="B10" s="58"/>
-      <c r="C10" s="58"/>
-      <c r="D10" s="59"/>
-      <c r="E10" s="60">
-        <f>SUM(G7:G9)</f>
-        <v>0</v>
-      </c>
-      <c r="F10" s="61"/>
-      <c r="G10" s="62"/>
-      <c r="H10" s="63">
-        <f>SUM(J7:J9)</f>
-        <v>0</v>
-      </c>
-      <c r="I10" s="61"/>
-      <c r="J10" s="62"/>
-      <c r="K10" s="63">
-        <f>SUM(M7:M9)</f>
-        <v>0</v>
-      </c>
-      <c r="L10" s="61"/>
-      <c r="M10" s="64"/>
-      <c r="N10" s="63">
-        <f>SUM(P7:P9)</f>
-        <v>0</v>
-      </c>
-      <c r="O10" s="61"/>
-      <c r="P10" s="64"/>
-      <c r="Q10" s="63">
-        <f>SUM(S7:S9)</f>
-        <v>0</v>
-      </c>
-      <c r="R10" s="61"/>
-      <c r="S10" s="64"/>
+      <c r="A10" s="52">
+        <v>4</v>
+      </c>
+      <c r="B10" s="53"/>
+      <c r="C10" s="53"/>
+      <c r="D10" s="53"/>
+      <c r="E10" s="50"/>
+      <c r="F10" s="50"/>
+      <c r="G10" s="50">
+        <f>IF(F10&gt;0,C10*F10,IF(E10&gt;0,C10*E10,0))</f>
+        <v>0</v>
+      </c>
+      <c r="H10" s="50"/>
+      <c r="I10" s="50"/>
+      <c r="J10" s="50">
+        <f>IF(I10&gt;0,C10*I10,IF(H10&gt;0,C10*H10,0))</f>
+        <v>0</v>
+      </c>
+      <c r="K10" s="50"/>
+      <c r="L10" s="50"/>
+      <c r="M10" s="50">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N10" s="50"/>
+      <c r="O10" s="50"/>
+      <c r="P10" s="50">
+        <f>IF(O10&gt;0,C10*O10,IF(N10&gt;0,C10*N10,0))</f>
+        <v>0</v>
+      </c>
+      <c r="Q10" s="50"/>
+      <c r="R10" s="50"/>
+      <c r="S10" s="51">
+        <f>IF(R10&gt;0,C10*R10,IF(Q10&gt;0,C10*Q10,0))</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="11" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A11" s="65" t="s">
-        <v>20</v>
-      </c>
-      <c r="B11" s="66"/>
-      <c r="C11" s="66"/>
-      <c r="D11" s="67"/>
-      <c r="E11" s="66"/>
-      <c r="F11" s="66"/>
-      <c r="G11" s="68"/>
-      <c r="H11" s="69"/>
-      <c r="I11" s="66"/>
-      <c r="J11" s="68"/>
-      <c r="K11" s="69"/>
-      <c r="L11" s="66"/>
-      <c r="M11" s="67"/>
-      <c r="N11" s="69"/>
-      <c r="O11" s="66"/>
-      <c r="P11" s="67"/>
-      <c r="Q11" s="69"/>
-      <c r="R11" s="66"/>
-      <c r="S11" s="67"/>
+      <c r="A11" s="52">
+        <v>5</v>
+      </c>
+      <c r="B11" s="53"/>
+      <c r="C11" s="53"/>
+      <c r="D11" s="53"/>
+      <c r="E11" s="54"/>
+      <c r="F11" s="54"/>
+      <c r="G11" s="54">
+        <f>IF(F11&gt;0,C11*F11,IF(E11&gt;0,C11*E11,0))</f>
+        <v>0</v>
+      </c>
+      <c r="H11" s="54"/>
+      <c r="I11" s="54"/>
+      <c r="J11" s="54">
+        <f>IF(I11&gt;0,C11*I11,IF(H11&gt;0,C11*H11,0))</f>
+        <v>0</v>
+      </c>
+      <c r="K11" s="54"/>
+      <c r="L11" s="54"/>
+      <c r="M11" s="54">
+        <f>IF(L11&gt;0,C11*L11,IF(K11&gt;0,C11*K11,0))</f>
+        <v>0</v>
+      </c>
+      <c r="N11" s="54"/>
+      <c r="O11" s="54"/>
+      <c r="P11" s="54">
+        <f>IF(O11&gt;0,C11*O11,IF(N11&gt;0,C11*N11,0))</f>
+        <v>0</v>
+      </c>
+      <c r="Q11" s="54"/>
+      <c r="R11" s="54"/>
+      <c r="S11" s="55">
+        <f>IF(R11&gt;0,C11*R11,IF(Q11&gt;0,C11*Q11,0))</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="12" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A12" s="70" t="s">
-        <v>21</v>
-      </c>
-      <c r="B12" s="71"/>
-      <c r="C12" s="71"/>
-      <c r="D12" s="72"/>
-      <c r="E12" s="73"/>
-      <c r="F12" s="73"/>
-      <c r="G12" s="74"/>
-      <c r="H12" s="75"/>
-      <c r="I12" s="73"/>
-      <c r="J12" s="74"/>
-      <c r="K12" s="75"/>
-      <c r="L12" s="73"/>
-      <c r="M12" s="76"/>
-      <c r="N12" s="75"/>
-      <c r="O12" s="73"/>
-      <c r="P12" s="76"/>
-      <c r="Q12" s="75"/>
-      <c r="R12" s="73"/>
-      <c r="S12" s="76"/>
+      <c r="A12" s="56" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="57"/>
+      <c r="C12" s="57"/>
+      <c r="D12" s="58"/>
+      <c r="E12" s="59">
+        <f>SUM(G7:G11)</f>
+        <v>0</v>
+      </c>
+      <c r="F12" s="60"/>
+      <c r="G12" s="61"/>
+      <c r="H12" s="62">
+        <f>SUM(J7:J11)</f>
+        <v>0</v>
+      </c>
+      <c r="I12" s="60"/>
+      <c r="J12" s="61"/>
+      <c r="K12" s="62">
+        <f>SUM(M7:M11)</f>
+        <v>0</v>
+      </c>
+      <c r="L12" s="60"/>
+      <c r="M12" s="63"/>
+      <c r="N12" s="62">
+        <f>SUM(P7:P11)</f>
+        <v>0</v>
+      </c>
+      <c r="O12" s="60"/>
+      <c r="P12" s="63"/>
+      <c r="Q12" s="62">
+        <f>SUM(S7:S11)</f>
+        <v>0</v>
+      </c>
+      <c r="R12" s="60"/>
+      <c r="S12" s="63"/>
     </row>
     <row r="13" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A13" s="77" t="s">
-        <v>22</v>
-      </c>
-      <c r="B13" s="78"/>
-      <c r="C13" s="78"/>
-      <c r="D13" s="79"/>
-      <c r="E13" s="80">
-        <f>SUM(E10:G12)</f>
-        <v>0</v>
-      </c>
-      <c r="F13" s="80"/>
-      <c r="G13" s="81"/>
-      <c r="H13" s="82">
-        <f>SUM(H10:J12)</f>
-        <v>0</v>
-      </c>
-      <c r="I13" s="80"/>
-      <c r="J13" s="81"/>
-      <c r="K13" s="82">
-        <f>SUM(K10:M12)</f>
-        <v>0</v>
-      </c>
-      <c r="L13" s="80"/>
-      <c r="M13" s="83"/>
-      <c r="N13" s="82">
-        <f>SUM(N10:P12)</f>
-        <v>0</v>
-      </c>
-      <c r="O13" s="80"/>
-      <c r="P13" s="83"/>
-      <c r="Q13" s="82">
-        <f>SUM(Q10:S12)</f>
-        <v>0</v>
-      </c>
-      <c r="R13" s="80"/>
-      <c r="S13" s="83"/>
+      <c r="A13" s="64" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="65"/>
+      <c r="C13" s="65"/>
+      <c r="D13" s="66"/>
+      <c r="E13" s="65"/>
+      <c r="F13" s="65"/>
+      <c r="G13" s="67"/>
+      <c r="H13" s="68"/>
+      <c r="I13" s="65"/>
+      <c r="J13" s="67"/>
+      <c r="K13" s="68"/>
+      <c r="L13" s="65"/>
+      <c r="M13" s="66"/>
+      <c r="N13" s="68"/>
+      <c r="O13" s="65"/>
+      <c r="P13" s="66"/>
+      <c r="Q13" s="68"/>
+      <c r="R13" s="65"/>
+      <c r="S13" s="66"/>
     </row>
     <row r="14" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A14" s="84" t="s">
-        <v>23</v>
-      </c>
-      <c r="B14" s="85"/>
-      <c r="C14" s="85"/>
-      <c r="D14" s="86"/>
-      <c r="E14" s="87"/>
-      <c r="F14" s="48"/>
-      <c r="G14" s="48"/>
-      <c r="H14" s="48"/>
-      <c r="I14" s="48"/>
-      <c r="J14" s="48"/>
-      <c r="K14" s="48"/>
-      <c r="L14" s="48"/>
-      <c r="M14" s="88"/>
-      <c r="N14" s="48"/>
-      <c r="O14" s="48"/>
-      <c r="P14" s="88"/>
-      <c r="Q14" s="48"/>
-      <c r="R14" s="48"/>
-      <c r="S14" s="88"/>
+      <c r="A14" s="69" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" s="70"/>
+      <c r="C14" s="70"/>
+      <c r="D14" s="71"/>
+      <c r="E14" s="72"/>
+      <c r="F14" s="72"/>
+      <c r="G14" s="73"/>
+      <c r="H14" s="74"/>
+      <c r="I14" s="72"/>
+      <c r="J14" s="73"/>
+      <c r="K14" s="74"/>
+      <c r="L14" s="72"/>
+      <c r="M14" s="75"/>
+      <c r="N14" s="74"/>
+      <c r="O14" s="72"/>
+      <c r="P14" s="75"/>
+      <c r="Q14" s="74"/>
+      <c r="R14" s="72"/>
+      <c r="S14" s="75"/>
     </row>
     <row r="15" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A15" s="47" t="s">
-        <v>24</v>
-      </c>
-      <c r="B15" s="48"/>
-      <c r="C15" s="48"/>
-      <c r="D15" s="88"/>
-      <c r="E15" s="68"/>
-      <c r="F15" s="43"/>
-      <c r="G15" s="43"/>
-      <c r="H15" s="68"/>
-      <c r="I15" s="43"/>
-      <c r="J15" s="43"/>
-      <c r="K15" s="68"/>
-      <c r="L15" s="43"/>
-      <c r="M15" s="89"/>
-      <c r="N15" s="68"/>
-      <c r="O15" s="43"/>
-      <c r="P15" s="89"/>
-      <c r="Q15" s="68"/>
-      <c r="R15" s="43"/>
-      <c r="S15" s="89"/>
+      <c r="A15" s="76" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15" s="77"/>
+      <c r="C15" s="77"/>
+      <c r="D15" s="78"/>
+      <c r="E15" s="79">
+        <f>SUM(E12:G14)</f>
+        <v>0</v>
+      </c>
+      <c r="F15" s="79"/>
+      <c r="G15" s="80"/>
+      <c r="H15" s="81">
+        <f>SUM(H12:J14)</f>
+        <v>0</v>
+      </c>
+      <c r="I15" s="79"/>
+      <c r="J15" s="80"/>
+      <c r="K15" s="81">
+        <f>SUM(K12:M14)</f>
+        <v>0</v>
+      </c>
+      <c r="L15" s="79"/>
+      <c r="M15" s="82"/>
+      <c r="N15" s="81">
+        <f>SUM(N12:P14)</f>
+        <v>0</v>
+      </c>
+      <c r="O15" s="79"/>
+      <c r="P15" s="82"/>
+      <c r="Q15" s="81">
+        <f>SUM(Q12:S14)</f>
+        <v>0</v>
+      </c>
+      <c r="R15" s="79"/>
+      <c r="S15" s="82"/>
     </row>
     <row r="16" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A16" s="47" t="s">
-        <v>25</v>
-      </c>
-      <c r="B16" s="48"/>
-      <c r="C16" s="48"/>
-      <c r="D16" s="88"/>
-      <c r="E16" s="68"/>
-      <c r="F16" s="43"/>
-      <c r="G16" s="43"/>
-      <c r="H16" s="68"/>
-      <c r="I16" s="43"/>
-      <c r="J16" s="43"/>
-      <c r="K16" s="68"/>
-      <c r="L16" s="43"/>
-      <c r="M16" s="89"/>
-      <c r="N16" s="68"/>
-      <c r="O16" s="43"/>
-      <c r="P16" s="89"/>
-      <c r="Q16" s="68"/>
-      <c r="R16" s="43"/>
-      <c r="S16" s="89"/>
+      <c r="A16" s="83" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" s="84"/>
+      <c r="C16" s="84"/>
+      <c r="D16" s="85"/>
+      <c r="E16" s="86"/>
+      <c r="F16" s="49"/>
+      <c r="G16" s="49"/>
+      <c r="H16" s="49"/>
+      <c r="I16" s="49"/>
+      <c r="J16" s="49"/>
+      <c r="K16" s="49"/>
+      <c r="L16" s="49"/>
+      <c r="M16" s="87"/>
+      <c r="N16" s="49"/>
+      <c r="O16" s="49"/>
+      <c r="P16" s="87"/>
+      <c r="Q16" s="49"/>
+      <c r="R16" s="49"/>
+      <c r="S16" s="87"/>
     </row>
     <row r="17" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A17" s="65" t="s">
-        <v>26</v>
-      </c>
-      <c r="B17" s="66"/>
-      <c r="C17" s="66"/>
-      <c r="D17" s="67"/>
-      <c r="E17" s="68"/>
-      <c r="F17" s="43"/>
-      <c r="G17" s="43"/>
-      <c r="H17" s="68"/>
-      <c r="I17" s="43"/>
-      <c r="J17" s="43"/>
-      <c r="K17" s="48"/>
-      <c r="L17" s="48"/>
+      <c r="A17" s="48" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17" s="49"/>
+      <c r="C17" s="49"/>
+      <c r="D17" s="87"/>
+      <c r="E17" s="67"/>
+      <c r="F17" s="45"/>
+      <c r="G17" s="45"/>
+      <c r="H17" s="67"/>
+      <c r="I17" s="45"/>
+      <c r="J17" s="45"/>
+      <c r="K17" s="67"/>
+      <c r="L17" s="45"/>
       <c r="M17" s="88"/>
-      <c r="N17" s="48"/>
-      <c r="O17" s="48"/>
+      <c r="N17" s="67"/>
+      <c r="O17" s="45"/>
       <c r="P17" s="88"/>
-      <c r="Q17" s="48"/>
-      <c r="R17" s="48"/>
+      <c r="Q17" s="67"/>
+      <c r="R17" s="45"/>
       <c r="S17" s="88"/>
     </row>
     <row r="18" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A18" s="84" t="s">
-        <v>27</v>
-      </c>
-      <c r="B18" s="85"/>
-      <c r="C18" s="85"/>
-      <c r="D18" s="86"/>
-      <c r="E18" s="87"/>
-      <c r="F18" s="48"/>
-      <c r="G18" s="48"/>
-      <c r="H18" s="48"/>
-      <c r="I18" s="48"/>
-      <c r="J18" s="48"/>
-      <c r="K18" s="48"/>
-      <c r="L18" s="48"/>
+      <c r="A18" s="48" t="s">
+        <v>25</v>
+      </c>
+      <c r="B18" s="49"/>
+      <c r="C18" s="49"/>
+      <c r="D18" s="87"/>
+      <c r="E18" s="67"/>
+      <c r="F18" s="45"/>
+      <c r="G18" s="45"/>
+      <c r="H18" s="67"/>
+      <c r="I18" s="45"/>
+      <c r="J18" s="45"/>
+      <c r="K18" s="67"/>
+      <c r="L18" s="45"/>
       <c r="M18" s="88"/>
-      <c r="N18" s="48"/>
-      <c r="O18" s="48"/>
+      <c r="N18" s="67"/>
+      <c r="O18" s="45"/>
       <c r="P18" s="88"/>
-      <c r="Q18" s="48"/>
-      <c r="R18" s="48"/>
+      <c r="Q18" s="67"/>
+      <c r="R18" s="45"/>
       <c r="S18" s="88"/>
     </row>
     <row r="19" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A19" s="84" t="s">
-        <v>28</v>
-      </c>
-      <c r="B19" s="85"/>
-      <c r="C19" s="85"/>
-      <c r="D19" s="86"/>
-      <c r="E19" s="87"/>
-      <c r="F19" s="48"/>
-      <c r="G19" s="48"/>
-      <c r="H19" s="48"/>
-      <c r="I19" s="48"/>
-      <c r="J19" s="48"/>
-      <c r="K19" s="48"/>
-      <c r="L19" s="48"/>
-      <c r="M19" s="88"/>
-      <c r="N19" s="48"/>
-      <c r="O19" s="48"/>
-      <c r="P19" s="88"/>
-      <c r="Q19" s="48"/>
-      <c r="R19" s="48"/>
-      <c r="S19" s="88"/>
+      <c r="A19" s="64" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" s="65"/>
+      <c r="C19" s="65"/>
+      <c r="D19" s="66"/>
+      <c r="E19" s="67"/>
+      <c r="F19" s="45"/>
+      <c r="G19" s="45"/>
+      <c r="H19" s="67"/>
+      <c r="I19" s="45"/>
+      <c r="J19" s="45"/>
+      <c r="K19" s="49"/>
+      <c r="L19" s="49"/>
+      <c r="M19" s="87"/>
+      <c r="N19" s="49"/>
+      <c r="O19" s="49"/>
+      <c r="P19" s="87"/>
+      <c r="Q19" s="49"/>
+      <c r="R19" s="49"/>
+      <c r="S19" s="87"/>
     </row>
     <row r="20" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A20" s="84" t="s">
-        <v>29</v>
-      </c>
-      <c r="B20" s="85"/>
-      <c r="C20" s="85"/>
-      <c r="D20" s="86"/>
-      <c r="E20" s="87"/>
-      <c r="F20" s="48"/>
-      <c r="G20" s="48"/>
-      <c r="H20" s="48"/>
-      <c r="I20" s="48"/>
-      <c r="J20" s="48"/>
-      <c r="K20" s="48"/>
-      <c r="L20" s="48"/>
-      <c r="M20" s="88"/>
-      <c r="N20" s="48"/>
-      <c r="O20" s="48"/>
-      <c r="P20" s="88"/>
-      <c r="Q20" s="48"/>
-      <c r="R20" s="48"/>
-      <c r="S20" s="88"/>
+      <c r="A20" s="83" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" s="84"/>
+      <c r="C20" s="84"/>
+      <c r="D20" s="85"/>
+      <c r="E20" s="86"/>
+      <c r="F20" s="49"/>
+      <c r="G20" s="49"/>
+      <c r="H20" s="49"/>
+      <c r="I20" s="49"/>
+      <c r="J20" s="49"/>
+      <c r="K20" s="49"/>
+      <c r="L20" s="49"/>
+      <c r="M20" s="87"/>
+      <c r="N20" s="49"/>
+      <c r="O20" s="49"/>
+      <c r="P20" s="87"/>
+      <c r="Q20" s="49"/>
+      <c r="R20" s="49"/>
+      <c r="S20" s="87"/>
     </row>
     <row r="21" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A21" s="84" t="s">
+      <c r="A21" s="83" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="84"/>
+      <c r="C21" s="84"/>
+      <c r="D21" s="85"/>
+      <c r="E21" s="86"/>
+      <c r="F21" s="49"/>
+      <c r="G21" s="49"/>
+      <c r="H21" s="49"/>
+      <c r="I21" s="49"/>
+      <c r="J21" s="49"/>
+      <c r="K21" s="49"/>
+      <c r="L21" s="49"/>
+      <c r="M21" s="87"/>
+      <c r="N21" s="49"/>
+      <c r="O21" s="49"/>
+      <c r="P21" s="87"/>
+      <c r="Q21" s="49"/>
+      <c r="R21" s="49"/>
+      <c r="S21" s="87"/>
+    </row>
+    <row r="22" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
+      <c r="A22" s="83" t="s">
+        <v>29</v>
+      </c>
+      <c r="B22" s="84"/>
+      <c r="C22" s="84"/>
+      <c r="D22" s="85"/>
+      <c r="E22" s="86"/>
+      <c r="F22" s="49"/>
+      <c r="G22" s="49"/>
+      <c r="H22" s="49"/>
+      <c r="I22" s="49"/>
+      <c r="J22" s="49"/>
+      <c r="K22" s="49"/>
+      <c r="L22" s="49"/>
+      <c r="M22" s="87"/>
+      <c r="N22" s="49"/>
+      <c r="O22" s="49"/>
+      <c r="P22" s="87"/>
+      <c r="Q22" s="49"/>
+      <c r="R22" s="49"/>
+      <c r="S22" s="87"/>
+    </row>
+    <row r="23" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
+      <c r="A23" s="83" t="s">
         <v>23</v>
       </c>
-      <c r="B21" s="85"/>
-      <c r="C21" s="85"/>
-      <c r="D21" s="86"/>
-      <c r="E21" s="87"/>
-      <c r="F21" s="48"/>
-      <c r="G21" s="48"/>
-      <c r="H21" s="48"/>
-      <c r="I21" s="48"/>
-      <c r="J21" s="48"/>
-      <c r="K21" s="48"/>
-      <c r="L21" s="48"/>
-      <c r="M21" s="88"/>
-      <c r="N21" s="48"/>
-      <c r="O21" s="48"/>
-      <c r="P21" s="88"/>
-      <c r="Q21" s="48"/>
-      <c r="R21" s="48"/>
-      <c r="S21" s="88"/>
-    </row>
-    <row r="22" s="2" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A22" s="84" t="s">
-        <v>30</v>
-      </c>
-      <c r="B22" s="85"/>
-      <c r="C22" s="85"/>
-      <c r="D22" s="86"/>
-      <c r="E22" s="87"/>
-      <c r="F22" s="48"/>
-      <c r="G22" s="48"/>
-      <c r="H22" s="48"/>
-      <c r="I22" s="48"/>
-      <c r="J22" s="48"/>
-      <c r="K22" s="48"/>
-      <c r="L22" s="48"/>
-      <c r="M22" s="88"/>
-      <c r="N22" s="48"/>
-      <c r="O22" s="48"/>
-      <c r="P22" s="88"/>
-      <c r="Q22" s="48"/>
-      <c r="R22" s="48"/>
-      <c r="S22" s="88"/>
-    </row>
-    <row r="23" s="2" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A23" s="90" t="s">
-        <v>31</v>
-      </c>
-      <c r="B23" s="91"/>
-      <c r="C23" s="91"/>
-      <c r="D23" s="92"/>
-      <c r="E23" s="93"/>
-      <c r="F23" s="94"/>
-      <c r="G23" s="94"/>
-      <c r="H23" s="94"/>
-      <c r="I23" s="94"/>
-      <c r="J23" s="94"/>
-      <c r="K23" s="94"/>
-      <c r="L23" s="94"/>
-      <c r="M23" s="95"/>
-      <c r="N23" s="94"/>
-      <c r="O23" s="94"/>
-      <c r="P23" s="95"/>
-      <c r="Q23" s="94"/>
-      <c r="R23" s="94"/>
-      <c r="S23" s="95"/>
+      <c r="B23" s="84"/>
+      <c r="C23" s="84"/>
+      <c r="D23" s="85"/>
+      <c r="E23" s="86"/>
+      <c r="F23" s="49"/>
+      <c r="G23" s="49"/>
+      <c r="H23" s="49"/>
+      <c r="I23" s="49"/>
+      <c r="J23" s="49"/>
+      <c r="K23" s="49"/>
+      <c r="L23" s="49"/>
+      <c r="M23" s="87"/>
+      <c r="N23" s="49"/>
+      <c r="O23" s="49"/>
+      <c r="P23" s="87"/>
+      <c r="Q23" s="49"/>
+      <c r="R23" s="49"/>
+      <c r="S23" s="87"/>
     </row>
     <row r="24" s="2" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A24" s="90" t="s">
-        <v>32</v>
-      </c>
-      <c r="B24" s="91"/>
-      <c r="C24" s="91"/>
-      <c r="D24" s="92"/>
-      <c r="E24" s="93"/>
-      <c r="F24" s="94"/>
-      <c r="G24" s="94"/>
-      <c r="H24" s="94"/>
-      <c r="I24" s="94"/>
-      <c r="J24" s="94"/>
-      <c r="K24" s="94"/>
-      <c r="L24" s="94"/>
-      <c r="M24" s="95"/>
-      <c r="N24" s="94"/>
-      <c r="O24" s="94"/>
-      <c r="P24" s="95"/>
-      <c r="Q24" s="94"/>
-      <c r="R24" s="94"/>
-      <c r="S24" s="95"/>
+      <c r="A24" s="83" t="s">
+        <v>30</v>
+      </c>
+      <c r="B24" s="84"/>
+      <c r="C24" s="84"/>
+      <c r="D24" s="85"/>
+      <c r="E24" s="86"/>
+      <c r="F24" s="49"/>
+      <c r="G24" s="49"/>
+      <c r="H24" s="49"/>
+      <c r="I24" s="49"/>
+      <c r="J24" s="49"/>
+      <c r="K24" s="49"/>
+      <c r="L24" s="49"/>
+      <c r="M24" s="87"/>
+      <c r="N24" s="49"/>
+      <c r="O24" s="49"/>
+      <c r="P24" s="87"/>
+      <c r="Q24" s="49"/>
+      <c r="R24" s="49"/>
+      <c r="S24" s="87"/>
     </row>
     <row r="25" s="2" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A25" s="96" t="s">
+      <c r="A25" s="89" t="s">
+        <v>31</v>
+      </c>
+      <c r="B25" s="90"/>
+      <c r="C25" s="90"/>
+      <c r="D25" s="91"/>
+      <c r="E25" s="92"/>
+      <c r="F25" s="93"/>
+      <c r="G25" s="93"/>
+      <c r="H25" s="93"/>
+      <c r="I25" s="93"/>
+      <c r="J25" s="93"/>
+      <c r="K25" s="93"/>
+      <c r="L25" s="93"/>
+      <c r="M25" s="94"/>
+      <c r="N25" s="93"/>
+      <c r="O25" s="93"/>
+      <c r="P25" s="94"/>
+      <c r="Q25" s="93"/>
+      <c r="R25" s="93"/>
+      <c r="S25" s="94"/>
+    </row>
+    <row r="26" s="2" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
+      <c r="A26" s="89" t="s">
+        <v>32</v>
+      </c>
+      <c r="B26" s="90"/>
+      <c r="C26" s="90"/>
+      <c r="D26" s="91"/>
+      <c r="E26" s="92"/>
+      <c r="F26" s="93"/>
+      <c r="G26" s="93"/>
+      <c r="H26" s="93"/>
+      <c r="I26" s="93"/>
+      <c r="J26" s="93"/>
+      <c r="K26" s="93"/>
+      <c r="L26" s="93"/>
+      <c r="M26" s="94"/>
+      <c r="N26" s="93"/>
+      <c r="O26" s="93"/>
+      <c r="P26" s="94"/>
+      <c r="Q26" s="93"/>
+      <c r="R26" s="93"/>
+      <c r="S26" s="94"/>
+    </row>
+    <row r="27" s="2" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
+      <c r="A27" s="95" t="s">
         <v>33</v>
       </c>
-      <c r="B25" s="97"/>
-      <c r="C25" s="97"/>
-      <c r="D25" s="98"/>
-      <c r="E25" s="93"/>
-      <c r="F25" s="94"/>
-      <c r="G25" s="94"/>
-      <c r="H25" s="94"/>
-      <c r="I25" s="94"/>
-      <c r="J25" s="94"/>
-      <c r="K25" s="94"/>
-      <c r="L25" s="94"/>
-      <c r="M25" s="95"/>
-      <c r="N25" s="94"/>
-      <c r="O25" s="94"/>
-      <c r="P25" s="95"/>
-      <c r="Q25" s="94"/>
-      <c r="R25" s="94"/>
-      <c r="S25" s="95"/>
+      <c r="B27" s="96"/>
+      <c r="C27" s="96"/>
+      <c r="D27" s="97"/>
+      <c r="E27" s="98"/>
+      <c r="F27" s="99"/>
+      <c r="G27" s="99"/>
+      <c r="H27" s="99"/>
+      <c r="I27" s="99"/>
+      <c r="J27" s="99"/>
+      <c r="K27" s="99"/>
+      <c r="L27" s="99"/>
+      <c r="M27" s="100"/>
+      <c r="N27" s="99"/>
+      <c r="O27" s="99"/>
+      <c r="P27" s="100"/>
+      <c r="Q27" s="99"/>
+      <c r="R27" s="99"/>
+      <c r="S27" s="100"/>
     </row>
   </sheetData>
   <mergeCells count="115">
@@ -2961,18 +2992,6 @@
     <mergeCell ref="K5:M5"/>
     <mergeCell ref="N5:P5"/>
     <mergeCell ref="Q5:S5"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="E10:G10"/>
-    <mergeCell ref="H10:J10"/>
-    <mergeCell ref="K10:M10"/>
-    <mergeCell ref="N10:P10"/>
-    <mergeCell ref="Q10:S10"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="E11:G11"/>
-    <mergeCell ref="H11:J11"/>
-    <mergeCell ref="K11:M11"/>
-    <mergeCell ref="N11:P11"/>
-    <mergeCell ref="Q11:S11"/>
     <mergeCell ref="A12:D12"/>
     <mergeCell ref="E12:G12"/>
     <mergeCell ref="H12:J12"/>
@@ -3057,6 +3076,18 @@
     <mergeCell ref="K25:M25"/>
     <mergeCell ref="N25:P25"/>
     <mergeCell ref="Q25:S25"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="E26:G26"/>
+    <mergeCell ref="H26:J26"/>
+    <mergeCell ref="K26:M26"/>
+    <mergeCell ref="N26:P26"/>
+    <mergeCell ref="Q26:S26"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="E27:G27"/>
+    <mergeCell ref="H27:J27"/>
+    <mergeCell ref="K27:M27"/>
+    <mergeCell ref="N27:P27"/>
+    <mergeCell ref="Q27:S27"/>
     <mergeCell ref="A4:A6"/>
     <mergeCell ref="B4:B6"/>
     <mergeCell ref="C4:C6"/>

</xml_diff>

<commit_message>
Fix merged cell attribute error in comparison export and update row/column mappings for new format sheet
</commit_message>
<xml_diff>
--- a/Comparision Format Sheet.xlsx
+++ b/Comparision Format Sheet.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19185" windowHeight="7500"/>
+    <workbookView windowWidth="19185" windowHeight="6900"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="33">
   <si>
     <t>COMPARATIVE STATEMENT</t>
   </si>
@@ -50,6 +50,9 @@
     <t xml:space="preserve"> Material Description</t>
   </si>
   <si>
+    <t>Make / Brand Offered</t>
+  </si>
+  <si>
     <t>Qty</t>
   </si>
   <si>
@@ -69,12 +72,6 @@
   </si>
   <si>
     <t>Vendor E</t>
-  </si>
-  <si>
-    <t>Brand !</t>
-  </si>
-  <si>
-    <t>Brand!</t>
   </si>
   <si>
     <t>Rate R0</t>
@@ -331,7 +328,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="42">
+  <fills count="41">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -364,12 +361,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF4B7BE"/>
-        <bgColor rgb="FF2F5597"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FF00B0F0"/>
         <bgColor rgb="FF2F5597"/>
       </patternFill>
@@ -579,7 +570,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="66">
+  <borders count="62">
     <border>
       <left/>
       <right/>
@@ -917,46 +908,6 @@
       <bottom style="medium">
         <color auto="1"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -1410,7 +1361,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="58" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="54" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1422,119 +1373,119 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="59" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="59" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="60" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="55" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="55" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="56" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="61" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="13" borderId="62" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="13" borderId="61" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="14" borderId="63" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="64" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="65" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="57" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="58" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="57" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="59" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="60" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="61" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="101">
+  <cellXfs count="98">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1558,6 +1509,9 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1579,6 +1533,9 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1597,6 +1554,9 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1630,37 +1590,19 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1675,163 +1617,163 @@
     <xf numFmtId="181" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="4" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="4" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="4" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="181" fontId="4" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="181" fontId="4" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="4" fillId="8" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="4" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="4" fillId="8" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="181" fontId="4" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="181" fontId="4" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="181" fontId="4" fillId="9" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="181" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="181" fontId="4" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="181" fontId="4" fillId="9" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="181" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="4" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="4" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="4" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="3" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="3" fillId="8" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="3" fillId="8" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="3" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="181" fontId="4" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="181" fontId="4" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="181" fontId="4" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="181" fontId="4" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="181" fontId="3" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="181" fontId="3" fillId="9" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="181" fontId="3" fillId="9" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="181" fontId="3" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2180,20 +2122,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:S27"/>
+  <dimension ref="A1:T26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.2" style="1" customWidth="1"/>
     <col min="2" max="2" width="32.7142857142857" style="1" customWidth="1"/>
-    <col min="3" max="3" width="10.1428571428571" style="1" customWidth="1"/>
-    <col min="4" max="4" width="12.2857142857143" style="1" customWidth="1"/>
-    <col min="5" max="11" width="15.5809523809524" style="1" customWidth="1"/>
-    <col min="12" max="12" width="20.152380952381" style="1" customWidth="1"/>
-    <col min="13" max="19" width="15.5809523809524" style="1" customWidth="1"/>
-    <col min="20" max="16384" width="9" style="1"/>
+    <col min="3" max="3" width="26.1428571428571" style="1" customWidth="1"/>
+    <col min="4" max="4" width="10.1428571428571" style="1" customWidth="1"/>
+    <col min="5" max="5" width="12.2857142857143" style="1" customWidth="1"/>
+    <col min="6" max="12" width="15.5809523809524" style="1" customWidth="1"/>
+    <col min="13" max="13" width="20.152380952381" style="1" customWidth="1"/>
+    <col min="14" max="20" width="15.5809523809524" style="1" customWidth="1"/>
+    <col min="21" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" ht="38.75" customHeight="1" spans="1:19">
+    <row r="1" s="1" customFormat="1" ht="38.75" customHeight="1" spans="1:20">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -2214,884 +2157,877 @@
       <c r="P1" s="4"/>
       <c r="Q1" s="4"/>
       <c r="R1" s="4"/>
-      <c r="S1" s="5"/>
+      <c r="S1" s="4"/>
+      <c r="T1" s="5"/>
     </row>
-    <row r="2" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
+    <row r="2" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:20">
       <c r="A2" s="6" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="7"/>
       <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
       <c r="K2" s="9"/>
-      <c r="L2" s="10" t="s">
+      <c r="L2" s="10"/>
+      <c r="M2" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="M2" s="11"/>
-      <c r="N2" s="11"/>
-      <c r="O2" s="11"/>
-      <c r="P2" s="11"/>
-      <c r="Q2" s="11"/>
-      <c r="R2" s="11"/>
+      <c r="N2" s="12"/>
+      <c r="O2" s="12"/>
+      <c r="P2" s="12"/>
+      <c r="Q2" s="12"/>
+      <c r="R2" s="12"/>
       <c r="S2" s="12"/>
+      <c r="T2" s="13"/>
     </row>
-    <row r="3" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A3" s="13" t="s">
+    <row r="3" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:20">
+      <c r="A3" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="14"/>
-      <c r="C3" s="15"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="15"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="15"/>
-      <c r="J3" s="15"/>
-      <c r="K3" s="16"/>
-      <c r="L3" s="17" t="s">
+      <c r="B3" s="15"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="17"/>
+      <c r="F3" s="17"/>
+      <c r="G3" s="17"/>
+      <c r="H3" s="17"/>
+      <c r="I3" s="17"/>
+      <c r="J3" s="17"/>
+      <c r="K3" s="17"/>
+      <c r="L3" s="18"/>
+      <c r="M3" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="M3" s="18"/>
-      <c r="N3" s="18"/>
-      <c r="O3" s="18"/>
-      <c r="P3" s="18"/>
-      <c r="Q3" s="18"/>
-      <c r="R3" s="18"/>
-      <c r="S3" s="19"/>
+      <c r="N3" s="20"/>
+      <c r="O3" s="20"/>
+      <c r="P3" s="20"/>
+      <c r="Q3" s="20"/>
+      <c r="R3" s="20"/>
+      <c r="S3" s="20"/>
+      <c r="T3" s="21"/>
     </row>
-    <row r="4" s="1" customFormat="1" ht="31.25" customHeight="1" spans="1:19">
-      <c r="A4" s="20" t="s">
+    <row r="4" s="1" customFormat="1" ht="31.25" customHeight="1" spans="1:20">
+      <c r="A4" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="21" t="s">
+      <c r="B4" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="C4" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="22" t="s">
+      <c r="D4" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="23" t="s">
+      <c r="E4" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="F4" s="24"/>
-      <c r="G4" s="24"/>
-      <c r="H4" s="25" t="s">
+      <c r="F4" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="I4" s="24"/>
-      <c r="J4" s="26"/>
-      <c r="K4" s="27" t="s">
+      <c r="G4" s="27"/>
+      <c r="H4" s="27"/>
+      <c r="I4" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="L4" s="28"/>
-      <c r="M4" s="29"/>
-      <c r="N4" s="30" t="s">
+      <c r="J4" s="27"/>
+      <c r="K4" s="29"/>
+      <c r="L4" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="O4" s="28"/>
-      <c r="P4" s="29"/>
-      <c r="Q4" s="30" t="s">
+      <c r="M4" s="31"/>
+      <c r="N4" s="32"/>
+      <c r="O4" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="R4" s="28"/>
-      <c r="S4" s="29"/>
+      <c r="P4" s="31"/>
+      <c r="Q4" s="32"/>
+      <c r="R4" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="S4" s="31"/>
+      <c r="T4" s="32"/>
     </row>
-    <row r="5" s="1" customFormat="1" ht="31.25" customHeight="1" spans="1:19">
-      <c r="A5" s="31"/>
-      <c r="B5" s="32"/>
-      <c r="C5" s="32"/>
-      <c r="D5" s="33"/>
-      <c r="E5" s="34" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5" s="35"/>
-      <c r="G5" s="36"/>
-      <c r="H5" s="35" t="s">
+    <row r="5" s="1" customFormat="1" ht="37" customHeight="1" spans="1:20">
+      <c r="A5" s="34"/>
+      <c r="B5" s="35"/>
+      <c r="C5" s="36"/>
+      <c r="D5" s="35"/>
+      <c r="E5" s="37"/>
+      <c r="F5" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="I5" s="35"/>
-      <c r="J5" s="36"/>
-      <c r="K5" s="35" t="s">
+      <c r="G5" s="39" t="s">
+        <v>16</v>
+      </c>
+      <c r="H5" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="I5" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="L5" s="35"/>
-      <c r="M5" s="37"/>
-      <c r="N5" s="35" t="s">
+      <c r="J5" s="39" t="s">
+        <v>16</v>
+      </c>
+      <c r="K5" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="L5" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="O5" s="35"/>
-      <c r="P5" s="37"/>
-      <c r="Q5" s="35" t="s">
+      <c r="M5" s="39" t="s">
+        <v>16</v>
+      </c>
+      <c r="N5" s="40" t="s">
+        <v>17</v>
+      </c>
+      <c r="O5" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="R5" s="35"/>
-      <c r="S5" s="37"/>
+      <c r="P5" s="39" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q5" s="40" t="s">
+        <v>17</v>
+      </c>
+      <c r="R5" s="39" t="s">
+        <v>15</v>
+      </c>
+      <c r="S5" s="39" t="s">
+        <v>16</v>
+      </c>
+      <c r="T5" s="40" t="s">
+        <v>17</v>
+      </c>
     </row>
-    <row r="6" s="1" customFormat="1" ht="37" customHeight="1" spans="1:19">
-      <c r="A6" s="38"/>
-      <c r="B6" s="39"/>
-      <c r="C6" s="39"/>
-      <c r="D6" s="40"/>
-      <c r="E6" s="41" t="s">
-        <v>16</v>
-      </c>
-      <c r="F6" s="42" t="s">
-        <v>17</v>
-      </c>
-      <c r="G6" s="42" t="s">
+    <row r="6" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:20">
+      <c r="A6" s="41">
+        <v>1</v>
+      </c>
+      <c r="B6" s="42"/>
+      <c r="C6" s="42"/>
+      <c r="D6" s="42"/>
+      <c r="E6" s="42"/>
+      <c r="F6" s="43"/>
+      <c r="G6" s="43"/>
+      <c r="H6" s="43">
+        <f t="shared" ref="H6:H10" si="0">IF(G6&gt;0,D6*G6,IF(F6&gt;0,D6*F6,0))</f>
+        <v>0</v>
+      </c>
+      <c r="I6" s="43"/>
+      <c r="J6" s="43"/>
+      <c r="K6" s="43">
+        <f t="shared" ref="K6:K10" si="1">IF(J6&gt;0,D6*J6,IF(I6&gt;0,D6*I6,0))</f>
+        <v>0</v>
+      </c>
+      <c r="L6" s="43"/>
+      <c r="M6" s="43"/>
+      <c r="N6" s="43">
+        <f t="shared" ref="N6:N10" si="2">IF(M6&gt;0,D6*M6,IF(L6&gt;0,D6*L6,0))</f>
+        <v>0</v>
+      </c>
+      <c r="O6" s="43"/>
+      <c r="P6" s="43"/>
+      <c r="Q6" s="43">
+        <f t="shared" ref="Q6:Q10" si="3">IF(P6&gt;0,D6*P6,IF(O6&gt;0,D6*O6,0))</f>
+        <v>0</v>
+      </c>
+      <c r="R6" s="43"/>
+      <c r="S6" s="43"/>
+      <c r="T6" s="44">
+        <f t="shared" ref="T6:T10" si="4">IF(S6&gt;0,D6*S6,IF(R6&gt;0,D6*R6,0))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:20">
+      <c r="A7" s="45">
+        <v>2</v>
+      </c>
+      <c r="B7" s="46"/>
+      <c r="C7" s="46"/>
+      <c r="D7" s="46"/>
+      <c r="E7" s="46"/>
+      <c r="F7" s="47"/>
+      <c r="G7" s="47"/>
+      <c r="H7" s="47">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I7" s="47"/>
+      <c r="J7" s="47"/>
+      <c r="K7" s="47">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="L7" s="47"/>
+      <c r="M7" s="47"/>
+      <c r="N7" s="47">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O7" s="47"/>
+      <c r="P7" s="47"/>
+      <c r="Q7" s="47">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="R7" s="47"/>
+      <c r="S7" s="47"/>
+      <c r="T7" s="48">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:20">
+      <c r="A8" s="49">
+        <v>3</v>
+      </c>
+      <c r="B8" s="50"/>
+      <c r="C8" s="50"/>
+      <c r="D8" s="50"/>
+      <c r="E8" s="50"/>
+      <c r="F8" s="47"/>
+      <c r="G8" s="47"/>
+      <c r="H8" s="47">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I8" s="47"/>
+      <c r="J8" s="47"/>
+      <c r="K8" s="47">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="L8" s="47"/>
+      <c r="M8" s="47"/>
+      <c r="N8" s="47">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O8" s="47"/>
+      <c r="P8" s="47"/>
+      <c r="Q8" s="47">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="R8" s="47"/>
+      <c r="S8" s="47"/>
+      <c r="T8" s="48">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:20">
+      <c r="A9" s="49">
+        <v>4</v>
+      </c>
+      <c r="B9" s="50"/>
+      <c r="C9" s="50"/>
+      <c r="D9" s="50"/>
+      <c r="E9" s="50"/>
+      <c r="F9" s="47"/>
+      <c r="G9" s="47"/>
+      <c r="H9" s="47">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I9" s="47"/>
+      <c r="J9" s="47"/>
+      <c r="K9" s="47">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="L9" s="47"/>
+      <c r="M9" s="47"/>
+      <c r="N9" s="47">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O9" s="47"/>
+      <c r="P9" s="47"/>
+      <c r="Q9" s="47">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="R9" s="47"/>
+      <c r="S9" s="47"/>
+      <c r="T9" s="48">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:20">
+      <c r="A10" s="49">
+        <v>5</v>
+      </c>
+      <c r="B10" s="50"/>
+      <c r="C10" s="50"/>
+      <c r="D10" s="50"/>
+      <c r="E10" s="50"/>
+      <c r="F10" s="51"/>
+      <c r="G10" s="51"/>
+      <c r="H10" s="51">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I10" s="51"/>
+      <c r="J10" s="51"/>
+      <c r="K10" s="51">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="L10" s="51"/>
+      <c r="M10" s="51"/>
+      <c r="N10" s="51">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O10" s="51"/>
+      <c r="P10" s="51"/>
+      <c r="Q10" s="51">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="R10" s="51"/>
+      <c r="S10" s="51"/>
+      <c r="T10" s="52">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:20">
+      <c r="A11" s="53" t="s">
         <v>18</v>
       </c>
-      <c r="H6" s="42" t="s">
-        <v>16</v>
-      </c>
-      <c r="I6" s="42" t="s">
-        <v>17</v>
-      </c>
-      <c r="J6" s="42" t="s">
-        <v>18</v>
-      </c>
-      <c r="K6" s="42" t="s">
-        <v>16</v>
-      </c>
-      <c r="L6" s="42" t="s">
-        <v>17</v>
-      </c>
-      <c r="M6" s="43" t="s">
-        <v>18</v>
-      </c>
-      <c r="N6" s="42" t="s">
-        <v>16</v>
-      </c>
-      <c r="O6" s="42" t="s">
-        <v>17</v>
-      </c>
-      <c r="P6" s="43" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q6" s="42" t="s">
-        <v>16</v>
-      </c>
-      <c r="R6" s="42" t="s">
-        <v>17</v>
-      </c>
-      <c r="S6" s="43" t="s">
-        <v>18</v>
-      </c>
+      <c r="B11" s="54"/>
+      <c r="C11" s="54"/>
+      <c r="D11" s="54"/>
+      <c r="E11" s="55"/>
+      <c r="F11" s="56">
+        <f>SUM(H6:H10)</f>
+        <v>0</v>
+      </c>
+      <c r="G11" s="57"/>
+      <c r="H11" s="58"/>
+      <c r="I11" s="59">
+        <f>SUM(K6:K10)</f>
+        <v>0</v>
+      </c>
+      <c r="J11" s="57"/>
+      <c r="K11" s="58"/>
+      <c r="L11" s="59">
+        <f>SUM(N6:N10)</f>
+        <v>0</v>
+      </c>
+      <c r="M11" s="57"/>
+      <c r="N11" s="60"/>
+      <c r="O11" s="59">
+        <f>SUM(Q6:Q10)</f>
+        <v>0</v>
+      </c>
+      <c r="P11" s="57"/>
+      <c r="Q11" s="60"/>
+      <c r="R11" s="59">
+        <f>SUM(T6:T10)</f>
+        <v>0</v>
+      </c>
+      <c r="S11" s="57"/>
+      <c r="T11" s="60"/>
     </row>
-    <row r="7" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A7" s="44">
-        <v>1</v>
-      </c>
-      <c r="B7" s="45"/>
-      <c r="C7" s="45"/>
-      <c r="D7" s="45"/>
-      <c r="E7" s="46"/>
-      <c r="F7" s="46"/>
-      <c r="G7" s="46">
-        <f t="shared" ref="G7:G9" si="0">IF(F7&gt;0,C7*F7,IF(E7&gt;0,C7*E7,0))</f>
-        <v>0</v>
-      </c>
-      <c r="H7" s="46"/>
-      <c r="I7" s="46"/>
-      <c r="J7" s="46">
-        <f t="shared" ref="J7:J9" si="1">IF(I7&gt;0,C7*I7,IF(H7&gt;0,C7*H7,0))</f>
-        <v>0</v>
-      </c>
-      <c r="K7" s="46"/>
-      <c r="L7" s="46"/>
-      <c r="M7" s="46">
-        <f t="shared" ref="M7:M10" si="2">IF(L7&gt;0,C7*L7,IF(K7&gt;0,C7*K7,0))</f>
-        <v>0</v>
-      </c>
-      <c r="N7" s="46"/>
-      <c r="O7" s="46"/>
-      <c r="P7" s="46">
-        <f t="shared" ref="P7:P9" si="3">IF(O7&gt;0,C7*O7,IF(N7&gt;0,C7*N7,0))</f>
-        <v>0</v>
-      </c>
-      <c r="Q7" s="46"/>
-      <c r="R7" s="46"/>
-      <c r="S7" s="47">
-        <f t="shared" ref="S7:S9" si="4">IF(R7&gt;0,C7*R7,IF(Q7&gt;0,C7*Q7,0))</f>
-        <v>0</v>
-      </c>
+    <row r="12" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:20">
+      <c r="A12" s="61" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="62"/>
+      <c r="C12" s="62"/>
+      <c r="D12" s="62"/>
+      <c r="E12" s="63"/>
+      <c r="F12" s="62"/>
+      <c r="G12" s="62"/>
+      <c r="H12" s="64"/>
+      <c r="I12" s="65"/>
+      <c r="J12" s="62"/>
+      <c r="K12" s="64"/>
+      <c r="L12" s="65"/>
+      <c r="M12" s="62"/>
+      <c r="N12" s="63"/>
+      <c r="O12" s="65"/>
+      <c r="P12" s="62"/>
+      <c r="Q12" s="63"/>
+      <c r="R12" s="65"/>
+      <c r="S12" s="62"/>
+      <c r="T12" s="63"/>
     </row>
-    <row r="8" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A8" s="48">
-        <v>2</v>
-      </c>
-      <c r="B8" s="49"/>
-      <c r="C8" s="49"/>
-      <c r="D8" s="49"/>
-      <c r="E8" s="50"/>
-      <c r="F8" s="50"/>
-      <c r="G8" s="50">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H8" s="50"/>
-      <c r="I8" s="50"/>
-      <c r="J8" s="50">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="K8" s="50"/>
-      <c r="L8" s="50"/>
-      <c r="M8" s="50">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="N8" s="50"/>
-      <c r="O8" s="50"/>
-      <c r="P8" s="50">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="Q8" s="50"/>
-      <c r="R8" s="50"/>
-      <c r="S8" s="51">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+    <row r="13" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:20">
+      <c r="A13" s="66" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="67"/>
+      <c r="C13" s="67"/>
+      <c r="D13" s="67"/>
+      <c r="E13" s="68"/>
+      <c r="F13" s="69"/>
+      <c r="G13" s="69"/>
+      <c r="H13" s="70"/>
+      <c r="I13" s="71"/>
+      <c r="J13" s="69"/>
+      <c r="K13" s="70"/>
+      <c r="L13" s="71"/>
+      <c r="M13" s="69"/>
+      <c r="N13" s="72"/>
+      <c r="O13" s="71"/>
+      <c r="P13" s="69"/>
+      <c r="Q13" s="72"/>
+      <c r="R13" s="71"/>
+      <c r="S13" s="69"/>
+      <c r="T13" s="72"/>
     </row>
-    <row r="9" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A9" s="52">
-        <v>3</v>
-      </c>
-      <c r="B9" s="53"/>
-      <c r="C9" s="53"/>
-      <c r="D9" s="53"/>
-      <c r="E9" s="50"/>
-      <c r="F9" s="50"/>
-      <c r="G9" s="50">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H9" s="50"/>
-      <c r="I9" s="50"/>
-      <c r="J9" s="50">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="K9" s="50"/>
-      <c r="L9" s="50"/>
-      <c r="M9" s="50">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="N9" s="50"/>
-      <c r="O9" s="50"/>
-      <c r="P9" s="50">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="Q9" s="50"/>
-      <c r="R9" s="50"/>
-      <c r="S9" s="51">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+    <row r="14" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:20">
+      <c r="A14" s="73" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" s="74"/>
+      <c r="C14" s="74"/>
+      <c r="D14" s="74"/>
+      <c r="E14" s="75"/>
+      <c r="F14" s="76">
+        <f>SUM(F11:H13)</f>
+        <v>0</v>
+      </c>
+      <c r="G14" s="76"/>
+      <c r="H14" s="77"/>
+      <c r="I14" s="78">
+        <f>SUM(I11:K13)</f>
+        <v>0</v>
+      </c>
+      <c r="J14" s="76"/>
+      <c r="K14" s="77"/>
+      <c r="L14" s="78">
+        <f>SUM(L11:N13)</f>
+        <v>0</v>
+      </c>
+      <c r="M14" s="76"/>
+      <c r="N14" s="79"/>
+      <c r="O14" s="78">
+        <f>SUM(O11:Q13)</f>
+        <v>0</v>
+      </c>
+      <c r="P14" s="76"/>
+      <c r="Q14" s="79"/>
+      <c r="R14" s="78">
+        <f>SUM(R11:T13)</f>
+        <v>0</v>
+      </c>
+      <c r="S14" s="76"/>
+      <c r="T14" s="79"/>
     </row>
-    <row r="10" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A10" s="52">
-        <v>4</v>
-      </c>
-      <c r="B10" s="53"/>
-      <c r="C10" s="53"/>
-      <c r="D10" s="53"/>
-      <c r="E10" s="50"/>
-      <c r="F10" s="50"/>
-      <c r="G10" s="50">
-        <f>IF(F10&gt;0,C10*F10,IF(E10&gt;0,C10*E10,0))</f>
-        <v>0</v>
-      </c>
-      <c r="H10" s="50"/>
-      <c r="I10" s="50"/>
-      <c r="J10" s="50">
-        <f>IF(I10&gt;0,C10*I10,IF(H10&gt;0,C10*H10,0))</f>
-        <v>0</v>
-      </c>
-      <c r="K10" s="50"/>
-      <c r="L10" s="50"/>
-      <c r="M10" s="50">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="N10" s="50"/>
-      <c r="O10" s="50"/>
-      <c r="P10" s="50">
-        <f>IF(O10&gt;0,C10*O10,IF(N10&gt;0,C10*N10,0))</f>
-        <v>0</v>
-      </c>
-      <c r="Q10" s="50"/>
-      <c r="R10" s="50"/>
-      <c r="S10" s="51">
-        <f>IF(R10&gt;0,C10*R10,IF(Q10&gt;0,C10*Q10,0))</f>
-        <v>0</v>
-      </c>
+    <row r="15" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:20">
+      <c r="A15" s="80" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15" s="81"/>
+      <c r="C15" s="81"/>
+      <c r="D15" s="81"/>
+      <c r="E15" s="82"/>
+      <c r="F15" s="83"/>
+      <c r="G15" s="46"/>
+      <c r="H15" s="46"/>
+      <c r="I15" s="46"/>
+      <c r="J15" s="46"/>
+      <c r="K15" s="46"/>
+      <c r="L15" s="46"/>
+      <c r="M15" s="46"/>
+      <c r="N15" s="84"/>
+      <c r="O15" s="46"/>
+      <c r="P15" s="46"/>
+      <c r="Q15" s="84"/>
+      <c r="R15" s="46"/>
+      <c r="S15" s="46"/>
+      <c r="T15" s="84"/>
     </row>
-    <row r="11" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A11" s="52">
-        <v>5</v>
-      </c>
-      <c r="B11" s="53"/>
-      <c r="C11" s="53"/>
-      <c r="D11" s="53"/>
-      <c r="E11" s="54"/>
-      <c r="F11" s="54"/>
-      <c r="G11" s="54">
-        <f>IF(F11&gt;0,C11*F11,IF(E11&gt;0,C11*E11,0))</f>
-        <v>0</v>
-      </c>
-      <c r="H11" s="54"/>
-      <c r="I11" s="54"/>
-      <c r="J11" s="54">
-        <f>IF(I11&gt;0,C11*I11,IF(H11&gt;0,C11*H11,0))</f>
-        <v>0</v>
-      </c>
-      <c r="K11" s="54"/>
-      <c r="L11" s="54"/>
-      <c r="M11" s="54">
-        <f>IF(L11&gt;0,C11*L11,IF(K11&gt;0,C11*K11,0))</f>
-        <v>0</v>
-      </c>
-      <c r="N11" s="54"/>
-      <c r="O11" s="54"/>
-      <c r="P11" s="54">
-        <f>IF(O11&gt;0,C11*O11,IF(N11&gt;0,C11*N11,0))</f>
-        <v>0</v>
-      </c>
-      <c r="Q11" s="54"/>
-      <c r="R11" s="54"/>
-      <c r="S11" s="55">
-        <f>IF(R11&gt;0,C11*R11,IF(Q11&gt;0,C11*Q11,0))</f>
-        <v>0</v>
-      </c>
+    <row r="16" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:20">
+      <c r="A16" s="45" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" s="46"/>
+      <c r="C16" s="46"/>
+      <c r="D16" s="46"/>
+      <c r="E16" s="84"/>
+      <c r="F16" s="64"/>
+      <c r="G16" s="42"/>
+      <c r="H16" s="42"/>
+      <c r="I16" s="64"/>
+      <c r="J16" s="42"/>
+      <c r="K16" s="42"/>
+      <c r="L16" s="64"/>
+      <c r="M16" s="42"/>
+      <c r="N16" s="85"/>
+      <c r="O16" s="64"/>
+      <c r="P16" s="42"/>
+      <c r="Q16" s="85"/>
+      <c r="R16" s="64"/>
+      <c r="S16" s="42"/>
+      <c r="T16" s="85"/>
     </row>
-    <row r="12" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A12" s="56" t="s">
-        <v>19</v>
-      </c>
-      <c r="B12" s="57"/>
-      <c r="C12" s="57"/>
-      <c r="D12" s="58"/>
-      <c r="E12" s="59">
-        <f>SUM(G7:G11)</f>
-        <v>0</v>
-      </c>
-      <c r="F12" s="60"/>
-      <c r="G12" s="61"/>
-      <c r="H12" s="62">
-        <f>SUM(J7:J11)</f>
-        <v>0</v>
-      </c>
-      <c r="I12" s="60"/>
-      <c r="J12" s="61"/>
-      <c r="K12" s="62">
-        <f>SUM(M7:M11)</f>
-        <v>0</v>
-      </c>
-      <c r="L12" s="60"/>
-      <c r="M12" s="63"/>
-      <c r="N12" s="62">
-        <f>SUM(P7:P11)</f>
-        <v>0</v>
-      </c>
-      <c r="O12" s="60"/>
-      <c r="P12" s="63"/>
-      <c r="Q12" s="62">
-        <f>SUM(S7:S11)</f>
-        <v>0</v>
-      </c>
-      <c r="R12" s="60"/>
-      <c r="S12" s="63"/>
+    <row r="17" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:20">
+      <c r="A17" s="45" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17" s="46"/>
+      <c r="C17" s="46"/>
+      <c r="D17" s="46"/>
+      <c r="E17" s="84"/>
+      <c r="F17" s="64"/>
+      <c r="G17" s="42"/>
+      <c r="H17" s="42"/>
+      <c r="I17" s="64"/>
+      <c r="J17" s="42"/>
+      <c r="K17" s="42"/>
+      <c r="L17" s="64"/>
+      <c r="M17" s="42"/>
+      <c r="N17" s="85"/>
+      <c r="O17" s="64"/>
+      <c r="P17" s="42"/>
+      <c r="Q17" s="85"/>
+      <c r="R17" s="64"/>
+      <c r="S17" s="42"/>
+      <c r="T17" s="85"/>
     </row>
-    <row r="13" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A13" s="64" t="s">
-        <v>20</v>
-      </c>
-      <c r="B13" s="65"/>
-      <c r="C13" s="65"/>
-      <c r="D13" s="66"/>
-      <c r="E13" s="65"/>
-      <c r="F13" s="65"/>
-      <c r="G13" s="67"/>
-      <c r="H13" s="68"/>
-      <c r="I13" s="65"/>
-      <c r="J13" s="67"/>
-      <c r="K13" s="68"/>
-      <c r="L13" s="65"/>
-      <c r="M13" s="66"/>
-      <c r="N13" s="68"/>
-      <c r="O13" s="65"/>
-      <c r="P13" s="66"/>
-      <c r="Q13" s="68"/>
-      <c r="R13" s="65"/>
-      <c r="S13" s="66"/>
+    <row r="18" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:20">
+      <c r="A18" s="61" t="s">
+        <v>25</v>
+      </c>
+      <c r="B18" s="62"/>
+      <c r="C18" s="62"/>
+      <c r="D18" s="62"/>
+      <c r="E18" s="63"/>
+      <c r="F18" s="64"/>
+      <c r="G18" s="42"/>
+      <c r="H18" s="42"/>
+      <c r="I18" s="64"/>
+      <c r="J18" s="42"/>
+      <c r="K18" s="42"/>
+      <c r="L18" s="46"/>
+      <c r="M18" s="46"/>
+      <c r="N18" s="84"/>
+      <c r="O18" s="46"/>
+      <c r="P18" s="46"/>
+      <c r="Q18" s="84"/>
+      <c r="R18" s="46"/>
+      <c r="S18" s="46"/>
+      <c r="T18" s="84"/>
     </row>
-    <row r="14" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A14" s="69" t="s">
-        <v>21</v>
-      </c>
-      <c r="B14" s="70"/>
-      <c r="C14" s="70"/>
-      <c r="D14" s="71"/>
-      <c r="E14" s="72"/>
-      <c r="F14" s="72"/>
-      <c r="G14" s="73"/>
-      <c r="H14" s="74"/>
-      <c r="I14" s="72"/>
-      <c r="J14" s="73"/>
-      <c r="K14" s="74"/>
-      <c r="L14" s="72"/>
-      <c r="M14" s="75"/>
-      <c r="N14" s="74"/>
-      <c r="O14" s="72"/>
-      <c r="P14" s="75"/>
-      <c r="Q14" s="74"/>
-      <c r="R14" s="72"/>
-      <c r="S14" s="75"/>
+    <row r="19" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:20">
+      <c r="A19" s="80" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" s="81"/>
+      <c r="C19" s="81"/>
+      <c r="D19" s="81"/>
+      <c r="E19" s="82"/>
+      <c r="F19" s="83"/>
+      <c r="G19" s="46"/>
+      <c r="H19" s="46"/>
+      <c r="I19" s="46"/>
+      <c r="J19" s="46"/>
+      <c r="K19" s="46"/>
+      <c r="L19" s="46"/>
+      <c r="M19" s="46"/>
+      <c r="N19" s="84"/>
+      <c r="O19" s="46"/>
+      <c r="P19" s="46"/>
+      <c r="Q19" s="84"/>
+      <c r="R19" s="46"/>
+      <c r="S19" s="46"/>
+      <c r="T19" s="84"/>
     </row>
-    <row r="15" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A15" s="76" t="s">
+    <row r="20" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:20">
+      <c r="A20" s="80" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" s="81"/>
+      <c r="C20" s="81"/>
+      <c r="D20" s="81"/>
+      <c r="E20" s="82"/>
+      <c r="F20" s="83"/>
+      <c r="G20" s="46"/>
+      <c r="H20" s="46"/>
+      <c r="I20" s="46"/>
+      <c r="J20" s="46"/>
+      <c r="K20" s="46"/>
+      <c r="L20" s="46"/>
+      <c r="M20" s="46"/>
+      <c r="N20" s="84"/>
+      <c r="O20" s="46"/>
+      <c r="P20" s="46"/>
+      <c r="Q20" s="84"/>
+      <c r="R20" s="46"/>
+      <c r="S20" s="46"/>
+      <c r="T20" s="84"/>
+    </row>
+    <row r="21" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:20">
+      <c r="A21" s="80" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="81"/>
+      <c r="C21" s="81"/>
+      <c r="D21" s="81"/>
+      <c r="E21" s="82"/>
+      <c r="F21" s="83"/>
+      <c r="G21" s="46"/>
+      <c r="H21" s="46"/>
+      <c r="I21" s="46"/>
+      <c r="J21" s="46"/>
+      <c r="K21" s="46"/>
+      <c r="L21" s="46"/>
+      <c r="M21" s="46"/>
+      <c r="N21" s="84"/>
+      <c r="O21" s="46"/>
+      <c r="P21" s="46"/>
+      <c r="Q21" s="84"/>
+      <c r="R21" s="46"/>
+      <c r="S21" s="46"/>
+      <c r="T21" s="84"/>
+    </row>
+    <row r="22" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:20">
+      <c r="A22" s="80" t="s">
         <v>22</v>
       </c>
-      <c r="B15" s="77"/>
-      <c r="C15" s="77"/>
-      <c r="D15" s="78"/>
-      <c r="E15" s="79">
-        <f>SUM(E12:G14)</f>
-        <v>0</v>
-      </c>
-      <c r="F15" s="79"/>
-      <c r="G15" s="80"/>
-      <c r="H15" s="81">
-        <f>SUM(H12:J14)</f>
-        <v>0</v>
-      </c>
-      <c r="I15" s="79"/>
-      <c r="J15" s="80"/>
-      <c r="K15" s="81">
-        <f>SUM(K12:M14)</f>
-        <v>0</v>
-      </c>
-      <c r="L15" s="79"/>
-      <c r="M15" s="82"/>
-      <c r="N15" s="81">
-        <f>SUM(N12:P14)</f>
-        <v>0</v>
-      </c>
-      <c r="O15" s="79"/>
-      <c r="P15" s="82"/>
-      <c r="Q15" s="81">
-        <f>SUM(Q12:S14)</f>
-        <v>0</v>
-      </c>
-      <c r="R15" s="79"/>
-      <c r="S15" s="82"/>
+      <c r="B22" s="81"/>
+      <c r="C22" s="81"/>
+      <c r="D22" s="81"/>
+      <c r="E22" s="82"/>
+      <c r="F22" s="83"/>
+      <c r="G22" s="46"/>
+      <c r="H22" s="46"/>
+      <c r="I22" s="46"/>
+      <c r="J22" s="46"/>
+      <c r="K22" s="46"/>
+      <c r="L22" s="46"/>
+      <c r="M22" s="46"/>
+      <c r="N22" s="84"/>
+      <c r="O22" s="46"/>
+      <c r="P22" s="46"/>
+      <c r="Q22" s="84"/>
+      <c r="R22" s="46"/>
+      <c r="S22" s="46"/>
+      <c r="T22" s="84"/>
     </row>
-    <row r="16" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A16" s="83" t="s">
-        <v>23</v>
-      </c>
-      <c r="B16" s="84"/>
-      <c r="C16" s="84"/>
-      <c r="D16" s="85"/>
-      <c r="E16" s="86"/>
-      <c r="F16" s="49"/>
-      <c r="G16" s="49"/>
-      <c r="H16" s="49"/>
-      <c r="I16" s="49"/>
-      <c r="J16" s="49"/>
-      <c r="K16" s="49"/>
-      <c r="L16" s="49"/>
-      <c r="M16" s="87"/>
-      <c r="N16" s="49"/>
-      <c r="O16" s="49"/>
-      <c r="P16" s="87"/>
-      <c r="Q16" s="49"/>
-      <c r="R16" s="49"/>
-      <c r="S16" s="87"/>
+    <row r="23" s="2" customFormat="1" ht="30.5" customHeight="1" spans="1:20">
+      <c r="A23" s="80" t="s">
+        <v>29</v>
+      </c>
+      <c r="B23" s="81"/>
+      <c r="C23" s="81"/>
+      <c r="D23" s="81"/>
+      <c r="E23" s="82"/>
+      <c r="F23" s="83"/>
+      <c r="G23" s="46"/>
+      <c r="H23" s="46"/>
+      <c r="I23" s="46"/>
+      <c r="J23" s="46"/>
+      <c r="K23" s="46"/>
+      <c r="L23" s="46"/>
+      <c r="M23" s="46"/>
+      <c r="N23" s="84"/>
+      <c r="O23" s="46"/>
+      <c r="P23" s="46"/>
+      <c r="Q23" s="84"/>
+      <c r="R23" s="46"/>
+      <c r="S23" s="46"/>
+      <c r="T23" s="84"/>
     </row>
-    <row r="17" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A17" s="48" t="s">
-        <v>24</v>
-      </c>
-      <c r="B17" s="49"/>
-      <c r="C17" s="49"/>
-      <c r="D17" s="87"/>
-      <c r="E17" s="67"/>
-      <c r="F17" s="45"/>
-      <c r="G17" s="45"/>
-      <c r="H17" s="67"/>
-      <c r="I17" s="45"/>
-      <c r="J17" s="45"/>
-      <c r="K17" s="67"/>
-      <c r="L17" s="45"/>
-      <c r="M17" s="88"/>
-      <c r="N17" s="67"/>
-      <c r="O17" s="45"/>
-      <c r="P17" s="88"/>
-      <c r="Q17" s="67"/>
-      <c r="R17" s="45"/>
-      <c r="S17" s="88"/>
+    <row r="24" s="2" customFormat="1" ht="30.5" customHeight="1" spans="1:20">
+      <c r="A24" s="86" t="s">
+        <v>30</v>
+      </c>
+      <c r="B24" s="87"/>
+      <c r="C24" s="87"/>
+      <c r="D24" s="87"/>
+      <c r="E24" s="88"/>
+      <c r="F24" s="89"/>
+      <c r="G24" s="90"/>
+      <c r="H24" s="90"/>
+      <c r="I24" s="90"/>
+      <c r="J24" s="90"/>
+      <c r="K24" s="90"/>
+      <c r="L24" s="90"/>
+      <c r="M24" s="90"/>
+      <c r="N24" s="91"/>
+      <c r="O24" s="90"/>
+      <c r="P24" s="90"/>
+      <c r="Q24" s="91"/>
+      <c r="R24" s="90"/>
+      <c r="S24" s="90"/>
+      <c r="T24" s="91"/>
     </row>
-    <row r="18" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A18" s="48" t="s">
-        <v>25</v>
-      </c>
-      <c r="B18" s="49"/>
-      <c r="C18" s="49"/>
-      <c r="D18" s="87"/>
-      <c r="E18" s="67"/>
-      <c r="F18" s="45"/>
-      <c r="G18" s="45"/>
-      <c r="H18" s="67"/>
-      <c r="I18" s="45"/>
-      <c r="J18" s="45"/>
-      <c r="K18" s="67"/>
-      <c r="L18" s="45"/>
-      <c r="M18" s="88"/>
-      <c r="N18" s="67"/>
-      <c r="O18" s="45"/>
-      <c r="P18" s="88"/>
-      <c r="Q18" s="67"/>
-      <c r="R18" s="45"/>
-      <c r="S18" s="88"/>
+    <row r="25" s="2" customFormat="1" ht="30.5" customHeight="1" spans="1:20">
+      <c r="A25" s="86" t="s">
+        <v>31</v>
+      </c>
+      <c r="B25" s="87"/>
+      <c r="C25" s="87"/>
+      <c r="D25" s="87"/>
+      <c r="E25" s="88"/>
+      <c r="F25" s="89"/>
+      <c r="G25" s="90"/>
+      <c r="H25" s="90"/>
+      <c r="I25" s="90"/>
+      <c r="J25" s="90"/>
+      <c r="K25" s="90"/>
+      <c r="L25" s="90"/>
+      <c r="M25" s="90"/>
+      <c r="N25" s="91"/>
+      <c r="O25" s="90"/>
+      <c r="P25" s="90"/>
+      <c r="Q25" s="91"/>
+      <c r="R25" s="90"/>
+      <c r="S25" s="90"/>
+      <c r="T25" s="91"/>
     </row>
-    <row r="19" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A19" s="64" t="s">
-        <v>26</v>
-      </c>
-      <c r="B19" s="65"/>
-      <c r="C19" s="65"/>
-      <c r="D19" s="66"/>
-      <c r="E19" s="67"/>
-      <c r="F19" s="45"/>
-      <c r="G19" s="45"/>
-      <c r="H19" s="67"/>
-      <c r="I19" s="45"/>
-      <c r="J19" s="45"/>
-      <c r="K19" s="49"/>
-      <c r="L19" s="49"/>
-      <c r="M19" s="87"/>
-      <c r="N19" s="49"/>
-      <c r="O19" s="49"/>
-      <c r="P19" s="87"/>
-      <c r="Q19" s="49"/>
-      <c r="R19" s="49"/>
-      <c r="S19" s="87"/>
-    </row>
-    <row r="20" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A20" s="83" t="s">
-        <v>27</v>
-      </c>
-      <c r="B20" s="84"/>
-      <c r="C20" s="84"/>
-      <c r="D20" s="85"/>
-      <c r="E20" s="86"/>
-      <c r="F20" s="49"/>
-      <c r="G20" s="49"/>
-      <c r="H20" s="49"/>
-      <c r="I20" s="49"/>
-      <c r="J20" s="49"/>
-      <c r="K20" s="49"/>
-      <c r="L20" s="49"/>
-      <c r="M20" s="87"/>
-      <c r="N20" s="49"/>
-      <c r="O20" s="49"/>
-      <c r="P20" s="87"/>
-      <c r="Q20" s="49"/>
-      <c r="R20" s="49"/>
-      <c r="S20" s="87"/>
-    </row>
-    <row r="21" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A21" s="83" t="s">
-        <v>28</v>
-      </c>
-      <c r="B21" s="84"/>
-      <c r="C21" s="84"/>
-      <c r="D21" s="85"/>
-      <c r="E21" s="86"/>
-      <c r="F21" s="49"/>
-      <c r="G21" s="49"/>
-      <c r="H21" s="49"/>
-      <c r="I21" s="49"/>
-      <c r="J21" s="49"/>
-      <c r="K21" s="49"/>
-      <c r="L21" s="49"/>
-      <c r="M21" s="87"/>
-      <c r="N21" s="49"/>
-      <c r="O21" s="49"/>
-      <c r="P21" s="87"/>
-      <c r="Q21" s="49"/>
-      <c r="R21" s="49"/>
-      <c r="S21" s="87"/>
-    </row>
-    <row r="22" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A22" s="83" t="s">
-        <v>29</v>
-      </c>
-      <c r="B22" s="84"/>
-      <c r="C22" s="84"/>
-      <c r="D22" s="85"/>
-      <c r="E22" s="86"/>
-      <c r="F22" s="49"/>
-      <c r="G22" s="49"/>
-      <c r="H22" s="49"/>
-      <c r="I22" s="49"/>
-      <c r="J22" s="49"/>
-      <c r="K22" s="49"/>
-      <c r="L22" s="49"/>
-      <c r="M22" s="87"/>
-      <c r="N22" s="49"/>
-      <c r="O22" s="49"/>
-      <c r="P22" s="87"/>
-      <c r="Q22" s="49"/>
-      <c r="R22" s="49"/>
-      <c r="S22" s="87"/>
-    </row>
-    <row r="23" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A23" s="83" t="s">
-        <v>23</v>
-      </c>
-      <c r="B23" s="84"/>
-      <c r="C23" s="84"/>
-      <c r="D23" s="85"/>
-      <c r="E23" s="86"/>
-      <c r="F23" s="49"/>
-      <c r="G23" s="49"/>
-      <c r="H23" s="49"/>
-      <c r="I23" s="49"/>
-      <c r="J23" s="49"/>
-      <c r="K23" s="49"/>
-      <c r="L23" s="49"/>
-      <c r="M23" s="87"/>
-      <c r="N23" s="49"/>
-      <c r="O23" s="49"/>
-      <c r="P23" s="87"/>
-      <c r="Q23" s="49"/>
-      <c r="R23" s="49"/>
-      <c r="S23" s="87"/>
-    </row>
-    <row r="24" s="2" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A24" s="83" t="s">
-        <v>30</v>
-      </c>
-      <c r="B24" s="84"/>
-      <c r="C24" s="84"/>
-      <c r="D24" s="85"/>
-      <c r="E24" s="86"/>
-      <c r="F24" s="49"/>
-      <c r="G24" s="49"/>
-      <c r="H24" s="49"/>
-      <c r="I24" s="49"/>
-      <c r="J24" s="49"/>
-      <c r="K24" s="49"/>
-      <c r="L24" s="49"/>
-      <c r="M24" s="87"/>
-      <c r="N24" s="49"/>
-      <c r="O24" s="49"/>
-      <c r="P24" s="87"/>
-      <c r="Q24" s="49"/>
-      <c r="R24" s="49"/>
-      <c r="S24" s="87"/>
-    </row>
-    <row r="25" s="2" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A25" s="89" t="s">
-        <v>31</v>
-      </c>
-      <c r="B25" s="90"/>
-      <c r="C25" s="90"/>
-      <c r="D25" s="91"/>
-      <c r="E25" s="92"/>
-      <c r="F25" s="93"/>
-      <c r="G25" s="93"/>
-      <c r="H25" s="93"/>
-      <c r="I25" s="93"/>
-      <c r="J25" s="93"/>
-      <c r="K25" s="93"/>
-      <c r="L25" s="93"/>
-      <c r="M25" s="94"/>
-      <c r="N25" s="93"/>
-      <c r="O25" s="93"/>
-      <c r="P25" s="94"/>
-      <c r="Q25" s="93"/>
-      <c r="R25" s="93"/>
-      <c r="S25" s="94"/>
-    </row>
-    <row r="26" s="2" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A26" s="89" t="s">
+    <row r="26" s="2" customFormat="1" ht="30.5" customHeight="1" spans="1:20">
+      <c r="A26" s="92" t="s">
         <v>32</v>
       </c>
-      <c r="B26" s="90"/>
-      <c r="C26" s="90"/>
-      <c r="D26" s="91"/>
-      <c r="E26" s="92"/>
-      <c r="F26" s="93"/>
-      <c r="G26" s="93"/>
-      <c r="H26" s="93"/>
-      <c r="I26" s="93"/>
-      <c r="J26" s="93"/>
-      <c r="K26" s="93"/>
-      <c r="L26" s="93"/>
-      <c r="M26" s="94"/>
-      <c r="N26" s="93"/>
-      <c r="O26" s="93"/>
-      <c r="P26" s="94"/>
-      <c r="Q26" s="93"/>
-      <c r="R26" s="93"/>
-      <c r="S26" s="94"/>
-    </row>
-    <row r="27" s="2" customFormat="1" ht="30.5" customHeight="1" spans="1:19">
-      <c r="A27" s="95" t="s">
-        <v>33</v>
-      </c>
-      <c r="B27" s="96"/>
-      <c r="C27" s="96"/>
-      <c r="D27" s="97"/>
-      <c r="E27" s="98"/>
-      <c r="F27" s="99"/>
-      <c r="G27" s="99"/>
-      <c r="H27" s="99"/>
-      <c r="I27" s="99"/>
-      <c r="J27" s="99"/>
-      <c r="K27" s="99"/>
-      <c r="L27" s="99"/>
-      <c r="M27" s="100"/>
-      <c r="N27" s="99"/>
-      <c r="O27" s="99"/>
-      <c r="P27" s="100"/>
-      <c r="Q27" s="99"/>
-      <c r="R27" s="99"/>
-      <c r="S27" s="100"/>
+      <c r="B26" s="93"/>
+      <c r="C26" s="93"/>
+      <c r="D26" s="93"/>
+      <c r="E26" s="94"/>
+      <c r="F26" s="95"/>
+      <c r="G26" s="96"/>
+      <c r="H26" s="96"/>
+      <c r="I26" s="96"/>
+      <c r="J26" s="96"/>
+      <c r="K26" s="96"/>
+      <c r="L26" s="96"/>
+      <c r="M26" s="96"/>
+      <c r="N26" s="97"/>
+      <c r="O26" s="96"/>
+      <c r="P26" s="96"/>
+      <c r="Q26" s="97"/>
+      <c r="R26" s="96"/>
+      <c r="S26" s="96"/>
+      <c r="T26" s="97"/>
     </row>
   </sheetData>
-  <mergeCells count="115">
-    <mergeCell ref="A1:S1"/>
-    <mergeCell ref="B2:K2"/>
-    <mergeCell ref="M2:S2"/>
-    <mergeCell ref="B3:K3"/>
-    <mergeCell ref="M3:S3"/>
-    <mergeCell ref="E4:G4"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="K4:M4"/>
-    <mergeCell ref="N4:P4"/>
-    <mergeCell ref="Q4:S4"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="H5:J5"/>
-    <mergeCell ref="K5:M5"/>
-    <mergeCell ref="N5:P5"/>
-    <mergeCell ref="Q5:S5"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="E12:G12"/>
-    <mergeCell ref="H12:J12"/>
-    <mergeCell ref="K12:M12"/>
-    <mergeCell ref="N12:P12"/>
-    <mergeCell ref="Q12:S12"/>
-    <mergeCell ref="A13:D13"/>
-    <mergeCell ref="E13:G13"/>
-    <mergeCell ref="H13:J13"/>
-    <mergeCell ref="K13:M13"/>
-    <mergeCell ref="N13:P13"/>
-    <mergeCell ref="Q13:S13"/>
-    <mergeCell ref="A14:D14"/>
-    <mergeCell ref="E14:G14"/>
-    <mergeCell ref="H14:J14"/>
-    <mergeCell ref="K14:M14"/>
-    <mergeCell ref="N14:P14"/>
-    <mergeCell ref="Q14:S14"/>
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="E15:G15"/>
-    <mergeCell ref="H15:J15"/>
-    <mergeCell ref="K15:M15"/>
-    <mergeCell ref="N15:P15"/>
-    <mergeCell ref="Q15:S15"/>
-    <mergeCell ref="A16:D16"/>
-    <mergeCell ref="E16:G16"/>
-    <mergeCell ref="H16:J16"/>
-    <mergeCell ref="K16:M16"/>
-    <mergeCell ref="N16:P16"/>
-    <mergeCell ref="Q16:S16"/>
-    <mergeCell ref="A17:D17"/>
-    <mergeCell ref="E17:G17"/>
-    <mergeCell ref="H17:J17"/>
-    <mergeCell ref="K17:M17"/>
-    <mergeCell ref="N17:P17"/>
-    <mergeCell ref="Q17:S17"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="E18:G18"/>
-    <mergeCell ref="H18:J18"/>
-    <mergeCell ref="K18:M18"/>
-    <mergeCell ref="N18:P18"/>
-    <mergeCell ref="Q18:S18"/>
-    <mergeCell ref="A19:D19"/>
-    <mergeCell ref="E19:G19"/>
-    <mergeCell ref="H19:J19"/>
-    <mergeCell ref="K19:M19"/>
-    <mergeCell ref="N19:P19"/>
-    <mergeCell ref="Q19:S19"/>
-    <mergeCell ref="A20:D20"/>
-    <mergeCell ref="E20:G20"/>
-    <mergeCell ref="H20:J20"/>
-    <mergeCell ref="K20:M20"/>
-    <mergeCell ref="N20:P20"/>
-    <mergeCell ref="Q20:S20"/>
-    <mergeCell ref="A21:D21"/>
-    <mergeCell ref="E21:G21"/>
-    <mergeCell ref="H21:J21"/>
-    <mergeCell ref="K21:M21"/>
-    <mergeCell ref="N21:P21"/>
-    <mergeCell ref="Q21:S21"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="E22:G22"/>
-    <mergeCell ref="H22:J22"/>
-    <mergeCell ref="K22:M22"/>
-    <mergeCell ref="N22:P22"/>
-    <mergeCell ref="Q22:S22"/>
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="E23:G23"/>
-    <mergeCell ref="H23:J23"/>
-    <mergeCell ref="K23:M23"/>
-    <mergeCell ref="N23:P23"/>
-    <mergeCell ref="Q23:S23"/>
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="E24:G24"/>
-    <mergeCell ref="H24:J24"/>
-    <mergeCell ref="K24:M24"/>
-    <mergeCell ref="N24:P24"/>
-    <mergeCell ref="Q24:S24"/>
-    <mergeCell ref="A25:D25"/>
-    <mergeCell ref="E25:G25"/>
-    <mergeCell ref="H25:J25"/>
-    <mergeCell ref="K25:M25"/>
-    <mergeCell ref="N25:P25"/>
-    <mergeCell ref="Q25:S25"/>
-    <mergeCell ref="A26:D26"/>
-    <mergeCell ref="E26:G26"/>
-    <mergeCell ref="H26:J26"/>
-    <mergeCell ref="K26:M26"/>
-    <mergeCell ref="N26:P26"/>
-    <mergeCell ref="Q26:S26"/>
-    <mergeCell ref="A27:D27"/>
-    <mergeCell ref="E27:G27"/>
-    <mergeCell ref="H27:J27"/>
-    <mergeCell ref="K27:M27"/>
-    <mergeCell ref="N27:P27"/>
-    <mergeCell ref="Q27:S27"/>
-    <mergeCell ref="A4:A6"/>
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="C4:C6"/>
-    <mergeCell ref="D4:D6"/>
+  <mergeCells count="111">
+    <mergeCell ref="A1:T1"/>
+    <mergeCell ref="B2:L2"/>
+    <mergeCell ref="N2:T2"/>
+    <mergeCell ref="B3:L3"/>
+    <mergeCell ref="N3:T3"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="I4:K4"/>
+    <mergeCell ref="L4:N4"/>
+    <mergeCell ref="O4:Q4"/>
+    <mergeCell ref="R4:T4"/>
+    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="F11:H11"/>
+    <mergeCell ref="I11:K11"/>
+    <mergeCell ref="L11:N11"/>
+    <mergeCell ref="O11:Q11"/>
+    <mergeCell ref="R11:T11"/>
+    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="F12:H12"/>
+    <mergeCell ref="I12:K12"/>
+    <mergeCell ref="L12:N12"/>
+    <mergeCell ref="O12:Q12"/>
+    <mergeCell ref="R12:T12"/>
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="F13:H13"/>
+    <mergeCell ref="I13:K13"/>
+    <mergeCell ref="L13:N13"/>
+    <mergeCell ref="O13:Q13"/>
+    <mergeCell ref="R13:T13"/>
+    <mergeCell ref="A14:E14"/>
+    <mergeCell ref="F14:H14"/>
+    <mergeCell ref="I14:K14"/>
+    <mergeCell ref="L14:N14"/>
+    <mergeCell ref="O14:Q14"/>
+    <mergeCell ref="R14:T14"/>
+    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="F15:H15"/>
+    <mergeCell ref="I15:K15"/>
+    <mergeCell ref="L15:N15"/>
+    <mergeCell ref="O15:Q15"/>
+    <mergeCell ref="R15:T15"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="F16:H16"/>
+    <mergeCell ref="I16:K16"/>
+    <mergeCell ref="L16:N16"/>
+    <mergeCell ref="O16:Q16"/>
+    <mergeCell ref="R16:T16"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="F17:H17"/>
+    <mergeCell ref="I17:K17"/>
+    <mergeCell ref="L17:N17"/>
+    <mergeCell ref="O17:Q17"/>
+    <mergeCell ref="R17:T17"/>
+    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="F18:H18"/>
+    <mergeCell ref="I18:K18"/>
+    <mergeCell ref="L18:N18"/>
+    <mergeCell ref="O18:Q18"/>
+    <mergeCell ref="R18:T18"/>
+    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="F19:H19"/>
+    <mergeCell ref="I19:K19"/>
+    <mergeCell ref="L19:N19"/>
+    <mergeCell ref="O19:Q19"/>
+    <mergeCell ref="R19:T19"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="F20:H20"/>
+    <mergeCell ref="I20:K20"/>
+    <mergeCell ref="L20:N20"/>
+    <mergeCell ref="O20:Q20"/>
+    <mergeCell ref="R20:T20"/>
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="F21:H21"/>
+    <mergeCell ref="I21:K21"/>
+    <mergeCell ref="L21:N21"/>
+    <mergeCell ref="O21:Q21"/>
+    <mergeCell ref="R21:T21"/>
+    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="F22:H22"/>
+    <mergeCell ref="I22:K22"/>
+    <mergeCell ref="L22:N22"/>
+    <mergeCell ref="O22:Q22"/>
+    <mergeCell ref="R22:T22"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="F23:H23"/>
+    <mergeCell ref="I23:K23"/>
+    <mergeCell ref="L23:N23"/>
+    <mergeCell ref="O23:Q23"/>
+    <mergeCell ref="R23:T23"/>
+    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="F24:H24"/>
+    <mergeCell ref="I24:K24"/>
+    <mergeCell ref="L24:N24"/>
+    <mergeCell ref="O24:Q24"/>
+    <mergeCell ref="R24:T24"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="F25:H25"/>
+    <mergeCell ref="I25:K25"/>
+    <mergeCell ref="L25:N25"/>
+    <mergeCell ref="O25:Q25"/>
+    <mergeCell ref="R25:T25"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="F26:H26"/>
+    <mergeCell ref="I26:K26"/>
+    <mergeCell ref="L26:N26"/>
+    <mergeCell ref="O26:Q26"/>
+    <mergeCell ref="R26:T26"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:E5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>